<commit_message>
consistency fix for calculating beyond-DLS stocks, update plot functions
</commit_message>
<xml_diff>
--- a/input/cover_for_result_files.xlsx
+++ b/input/cover_for_result_files.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jstreeck\Documents\GitHub\DLS_new_repo\input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jstreeck\Documents\GitHub\DLSmaterialStocks\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C0B2D21-ED17-4838-AA43-40A257897684}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{103F556C-128F-42CD-883C-E71C2D4F9421}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-57720" yWindow="1395" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-45" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -438,7 +438,7 @@
     <t>Fig3_global_product</t>
   </si>
   <si>
-    <t>Global material stocks (at scale, by product) catering to existing DLS, beyond-DLS, as well as the DLS material stock gaps for scenario i (the values for beyond-DLS stocks might differ slightly from those in Fig3_global_material due to differing resulting negatives for 'materials' and 'materials + products' when combining existing DLS with economy-wide stocks - when these are removed, the sum of the stock changes slightly depending on where negatives occur and how large they are</t>
+    <t xml:space="preserve">Global material stocks (at scale, by product) catering to existing DLS, beyond-DLS, as well as the DLS material stock gaps for scenario i </t>
   </si>
 </sst>
 </file>

</xml_diff>